<commit_message>
fix(ayuda-memoria): agrega 7 expedientes OV-CM/2024 faltantes (OD 340-343, 347-349)
Esos 7 (OV-175,176,234,450,451,452,453/24 -- Ministerio de RREE notificando
autorizaciones consulares) nunca habían sido scrapeados a proyectos.json:
scraper_proyectos.py busca por ventana de fecha reciente de *ingreso* del
expediente, y estos ingresaron en 2024 -- recién ahora tuvieron dictamen
conjunto de Asuntos Constitucionales y quedaron con OD asignado (349/26
entre otros). generar_ordenes_dia_xlsx.py los salteaba en silencio por
falta de match en proyectos.json. Se los agrega a mano con los datos reales
del sitio (extracto, comisión) y se vuelve a correr el pipeline completo.
</commit_message>
<xml_diff>
--- a/ordenes_dia_2026.xlsx
+++ b/ordenes_dia_2026.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I67"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2420,7 +2420,7 @@
         <v>2026</v>
       </c>
       <c r="B53" t="n">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -2429,12 +2429,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>OV-357/26-CM</t>
+          <t>OV-453/24-CM</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>MINISTERIO DE RELACIONES EXTERIORES Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO, JUAN LUIS GONZALEZ LANDA, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO VICECONSUL HONORARIO DE LOS ESTADOS UNIDOS MEXICANOS, EN LA CIUDAD DE MENDOZA, PROVINCIA HOMONIMA, CON JURISDICCION EN LAS PROVINCIAS DE SAN JUAN Y SAN LUIS.</t>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO OSCAR ENRIQUE MARTIN, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE VICECÓNSUL HONORARIO DE ESPAÑA EN GRAL. PICO  LA PAMPA.</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2458,7 +2458,7 @@
         <v>2026</v>
       </c>
       <c r="B54" t="n">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -2467,12 +2467,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>OV-331/26-CM</t>
+          <t>OV-452/24-CM</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO JAVIER JOSE CALVIÑO, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CONSUL HONORARIO DE LA REPUBLICA DEMOCRATICA DE TIMOR-LESTE, EN LA CIUDAD DE SAN ISIDRO, PROV. DE BS. AS., CON CIRCUNSCRIPCIÓN CONSULAR EN TODO EL TERRITORIO NACIONAL.</t>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR LA CIUDADANA ARGENTINA FLAVIA LORENA SEAGE, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE VICECONSUL HONORARIA DE ESPAÑA EN PUERTO IGUAZU, MISIONES.</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2496,7 +2496,7 @@
         <v>2026</v>
       </c>
       <c r="B55" t="n">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -2505,12 +2505,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>OV-300/26-CM</t>
+          <t>OV-451/24-CM</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO RODOLFO ERNESTO CAFFARO KRAMER, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CONSUL HONORARIO DEL REINO DE CAMBOYA, EN LA CIUDAD AUTONÓMA DE BUENOS AIRES, CON CIRCUNSCRIPCIÓN CONSULAR EN TODO EL TERRITORIO NACIONAL.</t>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO JOSE CARLOS ARCAGNI, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CÓNSUL HONORARIO DE LETONIA, EN  CABA.</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2534,7 +2534,7 @@
         <v>2026</v>
       </c>
       <c r="B56" t="n">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -2543,12 +2543,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>OV-74/26-CM</t>
+          <t>OV-450/24-CM</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>MINISTERIO DE RELACIONES EXTERIORES Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO GERMAN ENRIQUE BÖTTGER, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CONSUL HONORARIO DE LA REP. FEDERAL DE ALEMANIA EN LA CIUDAD DE SAN MIGUEL DE TUCUMAN, CON CIRCUNSCRIPCION EN LAS PROVINCIAS DE CATAMARCA, SANTIAGO DEL ESTERO Y TUCUMAN.</t>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO JUAN CARLOS SCHROEDER, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CÓNSUL HONORARIO DE ALEMANIA EN NEUQUEN.</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2572,7 +2572,7 @@
         <v>2026</v>
       </c>
       <c r="B57" t="n">
-        <v>351</v>
+        <v>344</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -2581,12 +2581,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>OV-32/26-CM</t>
+          <t>OV-357/26-CM</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>MINISTERIO DE RELACIONES EXTERIORES Y CULTO: REMITE NOTA ENVIADA POR LA CIUDADANA ARGENTINA ORIANA LAURA FOSSATI, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO AGENTE CÓNSULAR ADJUNTO DEL CONSULADO DE LA REPUBLICA ITALIANA EN MAR DEL PLATA, PROV, DE BS.AS.</t>
+          <t>MINISTERIO DE RELACIONES EXTERIORES Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO, JUAN LUIS GONZALEZ LANDA, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO VICECONSUL HONORARIO DE LOS ESTADOS UNIDOS MEXICANOS, EN LA CIUDAD DE MENDOZA, PROVINCIA HOMONIMA, CON JURISDICCION EN LAS PROVINCIAS DE SAN JUAN Y SAN LUIS.</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2610,7 +2610,7 @@
         <v>2026</v>
       </c>
       <c r="B58" t="n">
-        <v>352</v>
+        <v>345</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -2619,12 +2619,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>OV-31/26-CM</t>
+          <t>OV-331/26-CM</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>MINISTERIO DE RELACIONES EXTERIORES Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO JORGE LUIS PEREZ ALATI, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CONSUL HONORARIO DE LA REPUBLICA DE SINGAPUR EN LA CIUDAD AUTONOMA DE BUENOS AIRES.</t>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO JAVIER JOSE CALVIÑO, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CONSUL HONORARIO DE LA REPUBLICA DEMOCRATICA DE TIMOR-LESTE, EN LA CIUDAD DE SAN ISIDRO, PROV. DE BS. AS., CON CIRCUNSCRIPCIÓN CONSULAR EN TODO EL TERRITORIO NACIONAL.</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2648,7 +2648,7 @@
         <v>2026</v>
       </c>
       <c r="B59" t="n">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -2657,17 +2657,17 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>PE-35/26-AC</t>
+          <t>OV-300/26-CM</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>MENSAJE N° 46/26 QUE SOLICITA ACUERDO PARA DESIGNAR VOCAL DE LA CAMARA NACIONAL DE APELACIONES EN LO PENAL ECONOMICO, SALA B,  AL DR. ALEJANDRO JAVIER CATANIA.</t>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO RODOLFO ERNESTO CAFFARO KRAMER, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CONSUL HONORARIO DEL REINO DE CAMBOYA, EN LA CIUDAD AUTONÓMA DE BUENOS AIRES, CON CIRCUNSCRIPCIÓN CONSULAR EN TODO EL TERRITORIO NACIONAL.</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>DE ACUERDOS -</t>
+          <t>DE ASUNTOS CONSTITUCIONALES -</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -2686,7 +2686,7 @@
         <v>2026</v>
       </c>
       <c r="B60" t="n">
-        <v>354</v>
+        <v>347</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -2695,17 +2695,17 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>PE-37/26-AC</t>
+          <t>OV-234/24-CM</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>MENSAJE N° 48/26 QUE SOLICITA ACUERDO PARA DESIGNAR VOCAL DE LA CAMARA NACIONAL DE APELACIONES EN LO PENAL ECONOMICO, SALA A, AL DR. JUAN PEDRO GALVAN GREENWAY.</t>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO RAUL ENRIQUE BURGOS, QUE SOLICITA AUTORIZACION PARA DESEMPEÑARSE COMO VICECONSUL HONORARIO DE ESPAÑA EN LA CDAD. DE SAN SALVADOR DE JUJUY.</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>DE ACUERDOS -</t>
+          <t>DE ASUNTOS CONSTITUCIONALES -</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -2724,7 +2724,7 @@
         <v>2026</v>
       </c>
       <c r="B61" t="n">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -2733,17 +2733,17 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>S-517/25-PL</t>
+          <t>OV-176/24-CM</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>DE ANGELI: PROYECTO DE LEY QUE INSTITUYE EL DIA 15 DE ABRIL DE CADA AÑO COMO EL "DIA NACIONAL DEL INMIGRANTE ALEMAN DEL VOLGA".</t>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO DANIEL AMADO, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CÓNSUL HONORARIO DE PORTUGAL EN LA CIUDAD DE COMODORO RIVADAVIA, PROV. DEL CHUBUT.</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>DE POBLACIÓN Y DESARROLLO  HUMANO - DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE ASUNTOS CONSTITUCIONALES -</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -2762,7 +2762,7 @@
         <v>2026</v>
       </c>
       <c r="B62" t="n">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -2771,17 +2771,17 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>S-697/25-PL</t>
+          <t>OV-175/24-CM</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>AVILA: PROYECTO DE LEY QUE INCORPORA EL ART. 4 BIS A SU SIMILAR 25.415- PROGRAMA DE DETECCION DE LA HIPOACUSIA-, RESPECTO DE INCORPORAR DIVERSAS ACCIONES EN EL AMBITO EDUCATIVO.</t>
+          <t>MINISTERIO DE RELACIONES EXTERIORES, COMERCIO INTERNACIONAL Y CULTO: REMITE NOTA ENVIADA POR LA CIUDADANA ARGENTINA CAROLINA PATRICIA KAHR PIRA, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CÓNSUL HONORARIO DE AUSTRIA EN LA CIUDAD DE MENDOZA.</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>DE POBLACIÓN Y DESARROLLO  HUMANO - DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE ASUNTOS CONSTITUCIONALES -</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -2800,7 +2800,7 @@
         <v>2026</v>
       </c>
       <c r="B63" t="n">
-        <v>357</v>
+        <v>350</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -2809,17 +2809,17 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>S-319/25-PL</t>
+          <t>OV-74/26-CM</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>HUALA: REPRODUCE PROYECTO DE LEY QUE INSTITUYE EL 2 DE MAYO DE CADA AÑO COMO "DIA NACIONAL PARA LA PREVENCION DEL BULLYING Y OTRAS FORMAS DE VIOLENCIA Y ACOSO ESCOLAR". (REF. S. 1243/23)</t>
+          <t>MINISTERIO DE RELACIONES EXTERIORES Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO GERMAN ENRIQUE BÖTTGER, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CONSUL HONORARIO DE LA REP. FEDERAL DE ALEMANIA EN LA CIUDAD DE SAN MIGUEL DE TUCUMAN, CON CIRCUNSCRIPCION EN LAS PROVINCIAS DE CATAMARCA, SANTIAGO DEL ESTERO Y TUCUMAN.</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>DE POBLACIÓN Y DESARROLLO  HUMANO - DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE ASUNTOS CONSTITUCIONALES -</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -2838,7 +2838,7 @@
         <v>2026</v>
       </c>
       <c r="B64" t="n">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -2847,17 +2847,17 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>S-404/26-PL</t>
+          <t>OV-32/26-CM</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>GADANO: PROYECTO DE LEY QUE INSTITUYE EL DIA 27 DE NOVIEMBRE DE CADA AÑO COMO "DIA DEL BASTON VERDE".</t>
+          <t>MINISTERIO DE RELACIONES EXTERIORES Y CULTO: REMITE NOTA ENVIADA POR LA CIUDADANA ARGENTINA ORIANA LAURA FOSSATI, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO AGENTE CÓNSULAR ADJUNTO DEL CONSULADO DE LA REPUBLICA ITALIANA EN MAR DEL PLATA, PROV, DE BS.AS.</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>DE POBLACIÓN Y DESARROLLO  HUMANO - DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE ASUNTOS CONSTITUCIONALES -</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -2876,7 +2876,7 @@
         <v>2026</v>
       </c>
       <c r="B65" t="n">
-        <v>359</v>
+        <v>352</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -2885,17 +2885,17 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>S-997/26-PL</t>
+          <t>OV-31/26-CM</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>AVILA: PROYECTO DE LEY QUE ESTABLECE EL TERCER JUEVES DE MARZO DE CADA AÑO COMO EL "DIA DE REFLEXIÓN CONTRA LA VIOLENCIA JUVENIL.</t>
+          <t>MINISTERIO DE RELACIONES EXTERIORES Y CULTO: REMITE NOTA ENVIADA POR EL CIUDADANO ARGENTINO JORGE LUIS PEREZ ALATI, POR LA CUAL SOLICITA AUTORIZACION PARA DESEMPEÑARSE EN EL CARGO DE CONSUL HONORARIO DE LA REPUBLICA DE SINGAPUR EN LA CIUDAD AUTONOMA DE BUENOS AIRES.</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>DE POBLACIÓN Y DESARROLLO  HUMANO - DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE ASUNTOS CONSTITUCIONALES -</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -2914,7 +2914,7 @@
         <v>2026</v>
       </c>
       <c r="B66" t="n">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -2923,17 +2923,17 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>PE-243/26-CE</t>
+          <t>PE-35/26-AC</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>JEFATURA DE GABINETE: COMUNICA EL "ACUERDO DE TRANSFERENCIA DE LA FUNCION JUDICIAL EN MATERIA CRIMINAL Y CORRECCIONAL DE MENORES DEL ÁMBITO NACIONAL A LA JUSTICIA DE LA CIUDAD AUTÓNOMA DE BUENOS AIRES", CELEBRADO EL 3 DE JULIO DE 2026.</t>
+          <t>MENSAJE N° 46/26 QUE SOLICITA ACUERDO PARA DESIGNAR VOCAL DE LA CAMARA NACIONAL DE APELACIONES EN LO PENAL ECONOMICO, SALA B,  AL DR. ALEJANDRO JAVIER CATANIA.</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>DE JUSTICIA Y ASUNTOS PENALES - DE PRESUPUESTO Y HACIENDA -</t>
+          <t>DE ACUERDOS -</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -2952,34 +2952,300 @@
         <v>2026</v>
       </c>
       <c r="B67" t="n">
+        <v>354</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>PE-37/26-AC</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>MENSAJE N° 48/26 QUE SOLICITA ACUERDO PARA DESIGNAR VOCAL DE LA CAMARA NACIONAL DE APELACIONES EN LO PENAL ECONOMICO, SALA A, AL DR. JUAN PEDRO GALVAN GREENWAY.</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>DE ACUERDOS -</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B68" t="n">
+        <v>355</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>S-517/25-PL</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>DE ANGELI: PROYECTO DE LEY QUE INSTITUYE EL DIA 15 DE ABRIL DE CADA AÑO COMO EL "DIA NACIONAL DEL INMIGRANTE ALEMAN DEL VOLGA".</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>DE POBLACIÓN Y DESARROLLO  HUMANO - DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B69" t="n">
+        <v>356</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>S-697/25-PL</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>AVILA: PROYECTO DE LEY QUE INCORPORA EL ART. 4 BIS A SU SIMILAR 25.415- PROGRAMA DE DETECCION DE LA HIPOACUSIA-, RESPECTO DE INCORPORAR DIVERSAS ACCIONES EN EL AMBITO EDUCATIVO.</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>DE POBLACIÓN Y DESARROLLO  HUMANO - DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B70" t="n">
+        <v>357</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>S-319/25-PL</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>HUALA: REPRODUCE PROYECTO DE LEY QUE INSTITUYE EL 2 DE MAYO DE CADA AÑO COMO "DIA NACIONAL PARA LA PREVENCION DEL BULLYING Y OTRAS FORMAS DE VIOLENCIA Y ACOSO ESCOLAR". (REF. S. 1243/23)</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>DE POBLACIÓN Y DESARROLLO  HUMANO - DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B71" t="n">
+        <v>358</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>S-404/26-PL</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>GADANO: PROYECTO DE LEY QUE INSTITUYE EL DIA 27 DE NOVIEMBRE DE CADA AÑO COMO "DIA DEL BASTON VERDE".</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>DE POBLACIÓN Y DESARROLLO  HUMANO - DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B72" t="n">
+        <v>359</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>S-997/26-PL</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>AVILA: PROYECTO DE LEY QUE ESTABLECE EL TERCER JUEVES DE MARZO DE CADA AÑO COMO EL "DIA DE REFLEXIÓN CONTRA LA VIOLENCIA JUVENIL.</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>DE POBLACIÓN Y DESARROLLO  HUMANO - DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B73" t="n">
+        <v>360</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>PE-243/26-CE</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>JEFATURA DE GABINETE: COMUNICA EL "ACUERDO DE TRANSFERENCIA DE LA FUNCION JUDICIAL EN MATERIA CRIMINAL Y CORRECCIONAL DE MENORES DEL ÁMBITO NACIONAL A LA JUSTICIA DE LA CIUDAD AUTÓNOMA DE BUENOS AIRES", CELEBRADO EL 3 DE JULIO DE 2026.</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>DE JUSTICIA Y ASUNTOS PENALES - DE PRESUPUESTO Y HACIENDA -</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B74" t="n">
         <v>361</v>
       </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
         <is>
           <t>PE-244/26-CE</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr">
+      <c r="E74" t="inlineStr">
         <is>
           <t>JEFATURA DE GABINETE: COMUNICA EL CUARTO CONVENIO DE TRANSFERENCIA PROGRESIVA DE COMPETENCIAS PENALES DE LA JUSTICIA NACIONAL AL PODER JUDICIAL DE LA CIUDAD AUTÓNOMA DE BUENOS AIRES", CELEBRADO EL 3 DE JULIO DE 2026</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr">
+      <c r="F74" t="inlineStr">
         <is>
           <t>DE JUSTICIA Y ASUNTOS PENALES - DE PRESUPUESTO Y HACIENDA -</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
         <is>
           <t>Descargar</t>
         </is>
@@ -3119,6 +3385,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I66" r:id="rId130"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId131"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I73" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I74" r:id="rId146"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualización automática 2026-09-11 05:46 UTC
</commit_message>
<xml_diff>
--- a/ordenes_dia_2026.xlsx
+++ b/ordenes_dia_2026.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I76"/>
+  <dimension ref="A1:I102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>ANEXO</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2995,7 +2995,7 @@
         <v>2026</v>
       </c>
       <c r="B68" t="n">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -3004,17 +3004,23 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>CD-21/25-PL</t>
+          <t>S-1271/25-PL
+S-1861/25-PL
+S-3/26-PL
+S-809/26-PL
+S-916/26-PL
+S-1035/26-PL
+S-1246/26-PL</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>PROYECTO DE LEY EN REVISION QUE DECLARA HEROE NACIONAL AL BRIGADIER ESTANISLAO LOPEZ "PATRIARCA DEL FEDERALISMO ARGENTINO" EN RECONOCIMIENTO A SU ACCIONAR EN DEFENSA DE LOS IDEALES FEDERALES Y REPUBLICANOS.</t>
+          <t>AVILA: PROYECTO DE LEY QUE MODIFICA SU SIMILAR 27.640 - BIOCOMBUSTIBLES-, RESPECTO DEL PORCENTAJE OBLIGATORIO DE BIODIESEL Y BIOETANOL EN EL GASOIL Y LA NAFTA.</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>DE DEFENSA NACIONAL - DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE MINERÍA, ENERGÍA Y COMBUSTIBLES -</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3033,7 +3039,7 @@
         <v>2026</v>
       </c>
       <c r="B69" t="n">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -3042,17 +3048,17 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>S-1040/26-PL</t>
+          <t>CD-21/25-PL</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>VALENZUELA: PROYECTO DE LEY QUE DECLARA FIESTA NACIONAL AL "FESTIVAL DEL FOLCLORE CORRENTINO", A REALIZARSE EN LA CDAD. DE SANTO TOME, PROV. DE CORRIENTES, EN EL MES DE DICIEMBRE DE CADA AÑO.</t>
+          <t>PROYECTO DE LEY EN REVISION QUE DECLARA HEROE NACIONAL AL BRIGADIER ESTANISLAO LOPEZ "PATRIARCA DEL FEDERALISMO ARGENTINO" EN RECONOCIMIENTO A SU ACCIONAR EN DEFENSA DE LOS IDEALES FEDERALES Y REPUBLICANOS.</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE DEFENSA NACIONAL - DE EDUCACIÓN Y CULTURA -</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3071,7 +3077,7 @@
         <v>2026</v>
       </c>
       <c r="B70" t="n">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -3080,12 +3086,12 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>S-1239/26-PL</t>
+          <t>S-1040/26-PL</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>COTO: PROYECTO DE LEY QUE INSTITUYE EL 3 DE MARZO DE CADA AÑO, COMO "DIA NACIONAL EN HONOR AL ALMIRANTE GUILLERMO BROWN".</t>
+          <t>VALENZUELA: PROYECTO DE LEY QUE DECLARA FIESTA NACIONAL AL "FESTIVAL DEL FOLCLORE CORRENTINO", A REALIZARSE EN LA CDAD. DE SANTO TOME, PROV. DE CORRIENTES, EN EL MES DE DICIEMBRE DE CADA AÑO.</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3109,66 +3115,66 @@
         <v>2026</v>
       </c>
       <c r="B71" t="n">
+        <v>365</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>S-1239/26-PL</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>COTO: PROYECTO DE LEY QUE INSTITUYE EL 3 DE MARZO DE CADA AÑO, COMO "DIA NACIONAL EN HONOR AL ALMIRANTE GUILLERMO BROWN".</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B72" t="n">
         <v>366</v>
       </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
         <is>
           <t>S-718/26-PL
 S-808/26-PL
 S-865/26-PL</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
+      <c r="E72" t="inlineStr">
         <is>
           <t>CAPITANICH: PROYECTO DE LEY QUE ESTABLECE UN MARCO REGULATORIO PARA LA EMISIÓN Y DESARROLLO DE ACTIVOS FINANCIEROS AMBIENTALES (AFA).</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr">
+      <c r="F72" t="inlineStr">
         <is>
           <t>DE LEGISLACIÓN GENERAL - DE AMBIENTE Y DESARROLLO SUSTENTABLE - DE PRESUPUESTO Y HACIENDA -</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>Descargar</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B72" t="n">
-        <v>367</v>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>CD-7/26-PL</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>PROYECTO DE LEY EN REVISION QUE MODIFICA LA CARTA ORGANICA DEL BANCO CENTRAL DE LA REPUBLICA ARGENTINA.</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>DE ECONOMÍA NACIONAL E INVERSIÓN - DE PRESUPUESTO Y HACIENDA -</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -3187,7 +3193,7 @@
         <v>2026</v>
       </c>
       <c r="B73" t="n">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -3196,17 +3202,17 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>S-1643/25-PL</t>
+          <t>CD-7/26-PL</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>VISCHI: REPRODUCE PROYECTO DE LEY QUE DECLARA BIEN HISTORICO NACIONAL, EN LOS TERMINOS DE LA LEY 12.665 Y S/M., AL INMUEBLE IDENTIFICADO COMO EX "HOTEL DE INMIGRANTES- EX OFICINAS DE PUENTES Y CAMINOS DE GOYA", SITO EN LA MANZANA N° 497, ENTRE LAS CALLES CAÁ GUAZU Y AV. SARMIENTO DE LA CIUDAD DE GOYA, PROV. DE CORRIENTES. (REF. S.1422/22)</t>
+          <t>PROYECTO DE LEY EN REVISION QUE MODIFICA LA CARTA ORGANICA DEL BANCO CENTRAL DE LA REPUBLICA ARGENTINA.</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>DE EDUCACIÓN Y CULTURA -</t>
+          <t>DE ECONOMÍA NACIONAL E INVERSIÓN - DE PRESUPUESTO Y HACIENDA -</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -3225,7 +3231,7 @@
         <v>2026</v>
       </c>
       <c r="B74" t="n">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -3234,12 +3240,12 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>S-124/26-PL</t>
+          <t>S-1643/25-PL</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>AVILA: PROYECTO DE LEY QUE DECLARA MONUMENTO HISTORICO NACIONAL AL CEMENTERIO OESTE DE SAN MIGUEL DE TUCUMAN, PROV. DE TUCUMAN.</t>
+          <t>VISCHI: REPRODUCE PROYECTO DE LEY QUE DECLARA BIEN HISTORICO NACIONAL, EN LOS TERMINOS DE LA LEY 12.665 Y S/M., AL INMUEBLE IDENTIFICADO COMO EX "HOTEL DE INMIGRANTES- EX OFICINAS DE PUENTES Y CAMINOS DE GOYA", SITO EN LA MANZANA N° 497, ENTRE LAS CALLES CAÁ GUAZU Y AV. SARMIENTO DE LA CIUDAD DE GOYA, PROV. DE CORRIENTES. (REF. S.1422/22)</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3263,7 +3269,7 @@
         <v>2026</v>
       </c>
       <c r="B75" t="n">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -3272,12 +3278,12 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>S-255/26-PL</t>
+          <t>S-124/26-PL</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>FAMA: REPRODUCE PROYECTO DE LEY QUE MODIFICA SU SIMILAR 26.206 -EDUCACION NACIONAL-  RESPECTO DE PROMOVER EL DESARROLLO DE LA EDUCACION EMOCIONAL. (REF. S. 752/22)</t>
+          <t>AVILA: PROYECTO DE LEY QUE DECLARA MONUMENTO HISTORICO NACIONAL AL CEMENTERIO OESTE DE SAN MIGUEL DE TUCUMAN, PROV. DE TUCUMAN.</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3301,34 +3307,1024 @@
         <v>2026</v>
       </c>
       <c r="B76" t="n">
+        <v>370</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>S-255/26-PL</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>FAMA: REPRODUCE PROYECTO DE LEY QUE MODIFICA SU SIMILAR 26.206 -EDUCACION NACIONAL-  RESPECTO DE PROMOVER EL DESARROLLO DE LA EDUCACION EMOCIONAL. (REF. S. 752/22)</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B77" t="n">
         <v>371</v>
       </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
         <is>
           <t>S-447/26-PL</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
+      <c r="E77" t="inlineStr">
         <is>
           <t>MENDOZA Y OTROS: REPRODUCE PROYECTO DE LEY QUE DECLARA PATRIMONIO INMATERIAL CULTURAL Y NATURAL DE LA NACION, EN LOS TERMINOS DE LA LEY 26.118, AL "CHAKU", PRACTICA ANCESTRAL INCAICA DE CAPTURA, ESQUILA Y LIBERACIÓN DE VICUÑAS. (REF. S. 830/24).</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="F77" t="inlineStr">
         <is>
           <t>DE EDUCACIÓN Y CULTURA -</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr">
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B78" t="n">
+        <v>372</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>CD-8/26-PL</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>PROYECTO DE LEY EN REVISION QUE MODIFICA LAS LEYES 11683 Y 27799 (T.O. 1998 Y S/M) RELATIVAS A LA MODALIDAD SIMPLIFICADA DE DECLARACION JURADA DEL IMPUESTO A LAS GANANCIAS Y EN MATERIA DE PRESCRIPCION TRIBUTARIA, Y 25.191 REFERENTE AL REGIMEN SANCIONATORIO.</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>DE JUSTICIA Y ASUNTOS PENALES - DE PRESUPUESTO Y HACIENDA -</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B79" t="n">
+        <v>373</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>S-336/25-PD</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>JUEZ: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS EL "PROYECTO INSTITUCIONAL DE CONVIVENCIA, UNA INVITACIÓN A INNOVAR- VALORES EN ACCIÓN-", PARA IMPLEMENTAR EN SUS NIVELES INICIAL, PRIMARIO Y SECUNDARIO, DISEÑADO POR EL COLEGIO "LA MERCED" DE LA CDAD. DE RIO CUARTO, PROV. DE CÓRDOBA.</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B80" t="n">
+        <v>374</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>S-837/25-PD</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ROJAS DECUT: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL PROGRAMA DE EDUCACION FINANCIERA "CUENTAS SANAS" DE LA FUNDACION MACRO.</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B81" t="n">
+        <v>375</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>S-1469/25-PD</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>HUALA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO Y RECONOCE A LA ESCRITORA OLGA LILIANA REINOSO POR SU TRAYECTORIA Y APORTE A LA CULTURA.</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA - DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B82" t="n">
+        <v>376</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>S-1577/25-PD</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LEWANDOWSKI: PROYECTO DE DECLARACION QUE EXPRESA BENEPLACITO POR LA TRAYECTORIA DEL MUSICO MIGUEL FIGUEROA Y SU CONJUNTO "AMANECER CAMPERO", CON LA DIFUSION DEL CHAMAME EN EL AMBITO NACIONAL E INTERNACIONAL.</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B83" t="n">
+        <v>377</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>S-1601/25-PD</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>FERNÁNDEZ SAGASTI: PROYECTO DE DECLARACION QUE DECLARA DE INTERES EL EVENTO "CONVINART", RECONOCIENDO SU APORTE A LA DIFUSION DE LA CULTURA, EL ARTE Y LA IDENTIDAD NACIONAL.</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B84" t="n">
+        <v>378</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>S-1799/25-PD</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LÓPEZ: PROYECTO DE DECLARACIÓN QUE RECONOCE COMO VALOR HISTORICO Y CULTURAL AL MONOLITO DE LOMA BLANCA, EN LA LOCALIDAD DE OLTA, PROV. DE LA RIOJA.</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B85" t="n">
+        <v>379</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>S-1987/25-PD</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>GALARETTO: PROYECTO DE DECLARACION QUE DECLARA DE INTERES CULTURAL Y EDUCATIVO LA OBRA "DANZAS, BAILES Y COSTUMBRES DEL LITORAL ARGENTINO" DE LOS AUTORES CLAUDIA L. GARCIA Y ENRIQUE A. PIÑEYRO PUBLICADA POR EDITORIAL AUTORES ARGENTINOS EN 2025.</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B86" t="n">
+        <v>381</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>S-709/26-PD</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>FERNÁNDEZ SAGASTI: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR EL SUBCAMPEONATO LOGRADO POR ALUMNOS DE LA PROV. DE MENDOZA, EN EL MUNDIAL DE ROBOTICA "FIRST TECH CHALLENGE 2026", ENTRE EL 15 Y 18 DE ABRIL DE 2026.</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B87" t="n">
+        <v>382</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>S-735/26-PD</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OLIVERA LUCERO: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS LA FERIA INTERNACIONAL DE ARTESANIAS DE SAN JUAN 2026, EN LA LOC. DE CHIMBAS, PROV. DE SAN JUAN, ENTRE EL 30 DE ABRIL Y EL 11 DE MAYO</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B88" t="n">
+        <v>383</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>S-892/26-PD</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>ABDALA: PROYECTO DE DECLARACION QUE ADHIERE AL DÍA DEL GRANADERO PUNTANO EN DEDICACIÓN AL "HÉROE DE CHANCAY" CON MOTIVO DEL 231º ANIVERSARIO DEL NACIMIENTO DEL CORONEL JUAN PASCUAL PRINGLES.</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B89" t="n">
+        <v>384</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>S-900/26-PD</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>MORENO: PROYECTO DE DECLARACION QUE DECLARA DE INTERÉS EL "III CONGRESO INTERNACIONAL DE TRABAJO SOCIAL FORENSE: TSF, CULTURAS DIGITALES Y EMANCIPACIÓN", ORGANIZADO POR LA UNIVERSIDAD CATÓLICA DE SALTA (UCASAL), EN LA CDAD. HOMÓNIMA, DEL 23 AL 25 DE SEPTIEMBRE DE 2026.</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B90" t="n">
+        <v>385</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>S-934/26-PD</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>VALENZUELA: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA FIESTA PROVINCIAL DEL LOCRO, EN LA CDAD. DE CURUZU CUATIA, PROV. DE CORRIENTES, A REALIZARSE DEL 10 AL 12 DE JULIO DE 2026.</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B91" t="n">
+        <v>386</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>S-2149/25-PD
+S-300/26-PD</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>CAPITANICH: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA BIENAL INTERNACIONAL DE ESCULTURAS DE CHACO 2026, A REALIZARSE EN LA CDAD. DE RESISTENCIA, DEL 11 AL 19 DE JULIO DE 2026.</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B92" t="n">
+        <v>387</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>S-935/26-PD</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>VALENZUELA: PROYECTO DE DECLARACION QUE DECLARA DE INTERES LA 60° EDICION DEL "FESTIVAL DEL FOLCLORE CORRENTINO" EN LA CDAD. DE SANTO TOME, PROV. DE CORRIENTES, A REALIZARSE DEL 4 AL  6 DE DICIEMBRE DE 2026.</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B93" t="n">
+        <v>388</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>S-1006/26-PD</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>MONTE DE OCA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLACITO POR EL 35° ANIVERSARIO DE LA JURA DE LA CONSTITUCION DE LA PROV. DE TIERRA DEL FUEGO, A.I.A.S., EL 1 DE JUNIO DE 2026.</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B94" t="n">
+        <v>389</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>S-1017/26-PD</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>SCHNEIDER: PROYECTO DE DECLARACION QUE EXPRESA BENEPLACITO POR LA SELECCIÓN DE LAS DOCENTES CHAQUEÑAS VANESA ANABEL MEZA Y GLORIA ARGENTINA CISNEROS, COMO SEMIFINALISTAS NACIONALES EN LA EDICION 2026 DEL PREMIO "DOCENTES QUE INSPIRAN".</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B95" t="n">
+        <v>390</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>S-1020/26-PD</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>PAOLTRONI Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA COMPOSICION ARTISTICA "MI BANDERA ES ARGENTINA", DEL CANTAUTOR Y DOCENTE DE MUSICA DIAMANTINO RUBEN DARIO GIMENEZ.</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B96" t="n">
+        <v>391</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>S-1037/26-PD</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>ARCE Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA CUARTA EDICION DEL CONGRESO INTERNACIONAL VETERINARIO DEL IGUAZU (CIVI), A REALIZARSE EN LA PROV. DE MISIONES, EL 2 Y 3 DE OCTUBRE DE 2026.</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B97" t="n">
+        <v>392</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>S-1038/26-PD</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>ROJAS DECUT Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES LA PROPUESTA DIOCESANA CONMEMORATIVA DE LOS 400 AÑOS DE LA LLEGADA DE LAS MISIONES JESUITICAS Y LOS 40 AÑOS DE LA DIOCESIS DE PUERTO IGUAZU.</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B98" t="n">
+        <v>393</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>S-1104/26-PD</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>KRONEBERGER: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS EL LIBRO "ARGENTINA METROPOLITANA: ANTECEDENTES Y DESAFÍOS HACIA UNA GOBERNANZA REGIONAL" PUBLICADO POR LA ASOCIACIÓN CIVIL CUIDADANÍA METROPOLITANA.</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B99" t="n">
+        <v>394</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>S-1122/26-PD</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>AVILA: PROYECTO DE DECLARACIÓN QUE EXPRESA BENEPLÁCITO POR LA PARTICIPACIÓN Y SELECCIÓN DEL DOCENTE VÍCTOR DANIEL ZANOTTA, DE LA LOC. DE DELFÍN GALLO, PROV. DE TUCUMÁN, COMO SEMIFINALISTA NACIONAL EN LA EDICIÓN 2026 DEL PREMIO "DOCENTES QUE INSPIRAN".</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B100" t="n">
+        <v>395</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>S-1029/26-PD</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>GUZMÁN CORAITA Y OTROS: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES AL MUSEO DIDACTICO DE LA GESTA GUEMESIANA Y GAUCHA, EN LA LOC. DE SAN LORENZO, PROV. DE SALTA.</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B101" t="n">
+        <v>396</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>S-1154/26-PD
+S-1166/26-PD</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>ATAUCHE: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERES EL NUEVO ANIVERSARIO DEL EXODO JUJEÑO, EL 23 DE AGOSTO DE 2026.</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Descargar</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B102" t="n">
+        <v>397</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>S-1165/26-PD</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>MOISES: PROYECTO DE DECLARACIÓN QUE DECLARA DE INTERÉS LA CONMEMORACION DEL 190° ANIVERSARIO DEL NATALICIO DE DOÑA JOSEFA DOMINGA "PEPA" BALCARCE Y SAN MARTIN, EL 14 DE JULIO DE 2026.</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>DE EDUCACIÓN Y CULTURA -</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
         <is>
           <t>Descargar</t>
         </is>
@@ -3486,6 +4482,58 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId148"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId149"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I79" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I82" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I84" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I85" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I86" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I87" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I88" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I89" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I90" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I91" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I92" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I93" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I94" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I95" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D96" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I96" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D97" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I97" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D98" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I98" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I99" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I100" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I101" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D102" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I102" r:id="rId202"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>